<commit_message>
update m/s and group 12
</commit_message>
<xml_diff>
--- a/runs_eval/signal_controller_benchmark_real/full_performance_comparison_real.xlsx
+++ b/runs_eval/signal_controller_benchmark_real/full_performance_comparison_real.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Travid\updated_worst_case_MARL\runs_eval\signal_controller_benchmark_real\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36EDCA7C-FDFF-43E0-930F-DBBAF6BBE11A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{453D295B-D11E-41E6-81CF-024554524ED1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="4188" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -1544,7 +1544,7 @@
         <v>55.278699074073963</v>
       </c>
       <c r="C15" s="1">
-        <f t="shared" ref="C15:Y15" si="8">AVERAGE(C3:C14)</f>
+        <f t="shared" ref="C15:X15" si="8">AVERAGE(C3:C14)</f>
         <v>15.68983333333331</v>
       </c>
       <c r="D15" s="1">

</xml_diff>